<commit_message>
feat(url-ingestion): add website URL analysis and grounded FAQ generation
</commit_message>
<xml_diff>
--- a/tests/test_results.xlsx
+++ b/tests/test_results.xlsx
@@ -229,6 +229,90 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Test Distribution by Category</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <pieChart>
+        <varyColors val="1"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Executive Summary'!C11</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Executive Summary'!$B$12:$B$20</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Executive Summary'!$C$12:$C$20</f>
+            </numRef>
+          </val>
+        </ser>
+        <firstSliceAng val="0"/>
+      </pieChart>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>8</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="3600000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -520,7 +604,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:J20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -546,7 +630,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Generated on 2026-10-26 08:24:07 | Offline AI (Qwen2.5 3B)</t>
+          <t>Generated on 2026-10-31 09:23:07 | Offline AI (Qwen2.5 3B)</t>
         </is>
       </c>
     </row>
@@ -581,12 +665,12 @@
     <row r="6">
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>40</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>40</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -596,7 +680,7 @@
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>99.8%</t>
+          <t>100.0%</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
@@ -654,10 +738,10 @@
         </is>
       </c>
       <c r="C12" s="8" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
@@ -671,7 +755,7 @@
       </c>
       <c r="G12" s="8" t="inlineStr">
         <is>
-          <t>23.52 ms</t>
+          <t>12.46 ms</t>
         </is>
       </c>
     </row>
@@ -682,10 +766,10 @@
         </is>
       </c>
       <c r="C13" s="8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D13" s="8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E13" s="9" t="inlineStr">
         <is>
@@ -706,7 +790,7 @@
     <row r="14">
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Verification Engine</t>
+          <t>Semantic Analysis</t>
         </is>
       </c>
       <c r="C14" s="8" t="n">
@@ -722,26 +806,26 @@
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
-          <t>99.2%</t>
+          <t>100.0%</t>
         </is>
       </c>
       <c r="G14" s="8" t="inlineStr">
         <is>
-          <t>0.3 ms</t>
+          <t>809.72 ms</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Deduplication Engine</t>
+          <t>Generator &amp; Question Types</t>
         </is>
       </c>
       <c r="C15" s="8" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D15" s="8" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
@@ -755,21 +839,21 @@
       </c>
       <c r="G15" s="8" t="inlineStr">
         <is>
-          <t>1.75 ms</t>
+          <t>1924.07 ms</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>Export Engine</t>
+          <t>Verification Engine</t>
         </is>
       </c>
       <c r="C16" s="8" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D16" s="8" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
@@ -783,40 +867,125 @@
       </c>
       <c r="G16" s="8" t="inlineStr">
         <is>
-          <t>24.27 ms</t>
+          <t>0.0 ms</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="7" t="inlineStr">
         <is>
+          <t>Deduplication Engine</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="D17" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>0.0 ms</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Export Engine</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>27.8 ms</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="7" t="inlineStr">
+        <is>
           <t>API &amp; Infrastructure</t>
         </is>
       </c>
-      <c r="C17" s="8" t="n">
+      <c r="C19" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="D17" s="8" t="n">
+      <c r="D19" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="E17" s="9" t="inlineStr">
-        <is>
-          <t>100.0%</t>
-        </is>
-      </c>
-      <c r="F17" s="9" t="inlineStr">
-        <is>
-          <t>100.0%</t>
-        </is>
-      </c>
-      <c r="G17" s="8" t="inlineStr">
-        <is>
-          <t>0.0 ms</t>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="F19" s="9" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>238.66 ms</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Web Ingestion Engine</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="D20" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>2.53 ms</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -826,11 +995,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:J45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="29" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
     <col width="50" customWidth="1" min="4" max="4"/>
     <col width="50" customWidth="1" min="5" max="5"/>
@@ -845,14 +1014,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>FAQForge Test Case Catalog &amp; Deterministic Verification Results</t>
+          <t>FAQForge Full Test Case Catalog &amp; Deterministic Verification Results</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Deterministic verification results covering extraction, chunking, grounding, deduplication, and export.</t>
+          <t>Detailed evaluation covering text ingestion, chunking, linguistic analysis, FAQ generation, and anti-hallucination verification.</t>
         </is>
       </c>
     </row>
@@ -952,7 +1121,7 @@
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
-          <t>3.47 ms</t>
+          <t>0.0 ms</t>
         </is>
       </c>
       <c r="J6" s="11" t="inlineStr">
@@ -1004,7 +1173,7 @@
       </c>
       <c r="I7" s="8" t="inlineStr">
         <is>
-          <t>89.58 ms</t>
+          <t>74.76 ms</t>
         </is>
       </c>
       <c r="J7" s="11" t="inlineStr">
@@ -1056,7 +1225,7 @@
       </c>
       <c r="I8" s="8" t="inlineStr">
         <is>
-          <t>1.01 ms</t>
+          <t>0.0 ms</t>
         </is>
       </c>
       <c r="J8" s="11" t="inlineStr">
@@ -1125,32 +1294,32 @@
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>Chunking &amp; Tokenization</t>
+          <t>Document Processing</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Sentence Boundary Preservation</t>
+          <t>Multi-Page Metadata Integrity</t>
         </is>
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
-          <t>Verifies semantic chunker splits text at period/punctuation boundaries without cutting mid-word.</t>
+          <t>Verifies that document extraction encapsulates page numbers, headings, and character indices.</t>
         </is>
       </c>
       <c r="E10" s="10" t="inlineStr">
         <is>
-          <t>4 complete sentences totaling 16 words with target_words=10</t>
+          <t>Structured text document</t>
         </is>
       </c>
       <c r="F10" s="10" t="inlineStr">
         <is>
-          <t>Chunks preserve sentence endings without mid-word cuts</t>
+          <t>pages list containing page_number=1 with headings and word count</t>
         </is>
       </c>
       <c r="G10" s="10" t="inlineStr">
         <is>
-          <t>Generated 2 chunks cleanly on sentence boundaries</t>
+          <t>Pages detected: 1, page_number verified</t>
         </is>
       </c>
       <c r="H10" s="9" t="inlineStr">
@@ -1177,32 +1346,32 @@
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>Chunking &amp; Tokenization</t>
+          <t>Document Processing</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Sliding Window Chunk Overlap</t>
+          <t>Empty Document Graceful Rejection</t>
         </is>
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>Verifies contextual continuity by ensuring sequential chunks share overlap words.</t>
+          <t>Verifies ValueError raised when empty document is submitted.</t>
         </is>
       </c>
       <c r="E11" s="10" t="inlineStr">
         <is>
-          <t>120-word paragraph with target_words=30 and overlap_words=10</t>
+          <t>Empty text file</t>
         </is>
       </c>
       <c r="F11" s="10" t="inlineStr">
         <is>
-          <t>Multiple chunks produced sharing context across chunk boundaries</t>
+          <t>Raise ValueError indicating document is empty</t>
         </is>
       </c>
       <c r="G11" s="10" t="inlineStr">
         <is>
-          <t>Generated 5 continuous overlapping chunks</t>
+          <t>Empty file correctly caught and reported</t>
         </is>
       </c>
       <c r="H11" s="9" t="inlineStr">
@@ -1234,27 +1403,27 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Empty Text Safe Handling</t>
+          <t>Sentence Boundary Preservation</t>
         </is>
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>Verifies chunker gracefully returns empty list for empty or whitespace-only documents.</t>
+          <t>Verifies semantic chunker splits text at punctuation boundaries without cutting words.</t>
         </is>
       </c>
       <c r="E12" s="10" t="inlineStr">
         <is>
-          <t>Whitespace-only string</t>
+          <t>4 complete sentences totaling 16 words</t>
         </is>
       </c>
       <c r="F12" s="10" t="inlineStr">
         <is>
-          <t>Empty list [] returned without exceptions</t>
+          <t>Chunks preserve sentence endings without mid-word cuts</t>
         </is>
       </c>
       <c r="G12" s="10" t="inlineStr">
         <is>
-          <t>Returned []</t>
+          <t>Generated 2 chunks cleanly on sentence boundaries</t>
         </is>
       </c>
       <c r="H12" s="9" t="inlineStr">
@@ -1281,37 +1450,37 @@
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>Verification Engine</t>
+          <t>Chunking &amp; Tokenization</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Verbatim Factual Grounding Verification</t>
+          <t>Sliding Window Chunk Overlap</t>
         </is>
       </c>
       <c r="D13" s="10" t="inlineStr">
         <is>
-          <t>Verifies that an answer derived directly from source passage is marked 'verified' with high confidence.</t>
+          <t>Verifies contextual continuity by ensuring sequential chunks share overlap words.</t>
         </is>
       </c>
       <c r="E13" s="10" t="inlineStr">
         <is>
-          <t>Passage: 'Chapter headings must be formatted in 14 pt bold t...'</t>
+          <t>120-word paragraph with target_words=30 and overlap_words=10</t>
         </is>
       </c>
       <c r="F13" s="10" t="inlineStr">
         <is>
-          <t>status: 'verified', confidence &gt;= 0.85, needs_review: False</t>
+          <t>Multiple chunks produced sharing context across chunk boundaries</t>
         </is>
       </c>
       <c r="G13" s="10" t="inlineStr">
         <is>
-          <t>status: 'verified', confidence: 0.99, excerpt located</t>
+          <t>Generated 5 continuous overlapping chunks</t>
         </is>
       </c>
       <c r="H13" s="9" t="inlineStr">
         <is>
-          <t>99.0%</t>
+          <t>100.0%</t>
         </is>
       </c>
       <c r="I13" s="8" t="inlineStr">
@@ -1333,32 +1502,32 @@
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>Verification Engine</t>
+          <t>Chunking &amp; Tokenization</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Hallucinated Numerical Detection</t>
+          <t>Ultra-Long Sentence Overflow Protection</t>
         </is>
       </c>
       <c r="D14" s="10" t="inlineStr">
         <is>
-          <t>Validates that when an answer introduces fictitious numbers not in source, verification flags it for review.</t>
+          <t>Verifies that an exceptionally long sentence is kept intact as a discrete chunk without dropping data.</t>
         </is>
       </c>
       <c r="E14" s="10" t="inlineStr">
         <is>
-          <t>Source: '12 months', Answer: '36 months' (hallucination)</t>
+          <t>120-word continuous sentence without internal punctuation</t>
         </is>
       </c>
       <c r="F14" s="10" t="inlineStr">
         <is>
-          <t>Flagged with needs_review=True due to unsupported numerical claim</t>
+          <t>Chunk preserved without truncation or data loss</t>
         </is>
       </c>
       <c r="G14" s="10" t="inlineStr">
         <is>
-          <t>Status: rejected, Reason: Answer contains numbers/dates not present in source: 36</t>
+          <t>Processed into 1 chunk(s), full content preserved</t>
         </is>
       </c>
       <c r="H14" s="9" t="inlineStr">
@@ -1385,32 +1554,32 @@
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>Verification Engine</t>
+          <t>Chunking &amp; Tokenization</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Out-of-Domain Hallucination Detection</t>
+          <t>Empty Text Safe Handling</t>
         </is>
       </c>
       <c r="D15" s="10" t="inlineStr">
         <is>
-          <t>Verifies that completely ungrounded answers are assigned low confidence and rejected.</t>
+          <t>Verifies chunker gracefully returns empty list for empty or whitespace-only documents.</t>
         </is>
       </c>
       <c r="E15" s="10" t="inlineStr">
         <is>
-          <t>Biology passage vs Cryptography answer</t>
+          <t>Whitespace-only string</t>
         </is>
       </c>
       <c r="F15" s="10" t="inlineStr">
         <is>
-          <t>status in ['rejected', 'needs_review'] with confidence &lt;= 0.40</t>
+          <t>Empty list [] returned without exceptions</t>
         </is>
       </c>
       <c r="G15" s="10" t="inlineStr">
         <is>
-          <t>status: 'rejected', confidence: 0.4</t>
+          <t>Returned []</t>
         </is>
       </c>
       <c r="H15" s="9" t="inlineStr">
@@ -1420,7 +1589,7 @@
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
-          <t>1.49 ms</t>
+          <t>0.0 ms</t>
         </is>
       </c>
       <c r="J15" s="11" t="inlineStr">
@@ -1437,37 +1606,37 @@
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>Verification Engine</t>
+          <t>Chunking &amp; Tokenization</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Morphological Root Alignment</t>
+          <t>Section Heading Inheritance in Chunks</t>
         </is>
       </c>
       <c r="D16" s="10" t="inlineStr">
         <is>
-          <t>Verifies that morphological variants (e.g. 'formatting' vs 'format', 'require' vs 'requirement') match roots.</t>
+          <t>Verifies that chunks created under a specific section heading inherit the section name.</t>
         </is>
       </c>
       <c r="E16" s="10" t="inlineStr">
         <is>
-          <t>Passage: 'format', Answer: 'formatting'</t>
+          <t>Document with 2 distinct section headings</t>
         </is>
       </c>
       <c r="F16" s="10" t="inlineStr">
         <is>
-          <t>Morphological match recognizes 'format'/'formatting' root</t>
+          <t>Chunks contain section metadata tags</t>
         </is>
       </c>
       <c r="G16" s="10" t="inlineStr">
         <is>
-          <t>Status: verified, Confidence: 0.97</t>
+          <t>Section mappings: ['Header B']</t>
         </is>
       </c>
       <c r="H16" s="9" t="inlineStr">
         <is>
-          <t>97.0%</t>
+          <t>100.0%</t>
         </is>
       </c>
       <c r="I16" s="8" t="inlineStr">
@@ -1489,32 +1658,32 @@
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>Verification Engine</t>
+          <t>Semantic Analysis</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>Empty Input Handling</t>
+          <t>spaCy Named Entity Recognition (NER)</t>
         </is>
       </c>
       <c r="D17" s="10" t="inlineStr">
         <is>
-          <t>Verifies that empty questions, answers, or contexts return status 'rejected' with 0.0 confidence.</t>
+          <t>Verifies extraction of DATE, ORG, and MONEY entities from technical documents.</t>
         </is>
       </c>
       <c r="E17" s="10" t="inlineStr">
         <is>
-          <t>Empty question, answer, and passage strings</t>
+          <t>Text with date, university, and grant amount</t>
         </is>
       </c>
       <c r="F17" s="10" t="inlineStr">
         <is>
-          <t>status: 'rejected', confidence: 0.0, needs_review: True</t>
+          <t>Extracted entities with DATE, ORG, or MONEY labels</t>
         </is>
       </c>
       <c r="G17" s="10" t="inlineStr">
         <is>
-          <t>status: 'rejected', confidence: 0.0</t>
+          <t>Detected entities: [('October 24, 2024', 'DATE'), ('Stanford University', 'ORG'), ('50,000', 'MONEY'), ('AI', 'ORG')]</t>
         </is>
       </c>
       <c r="H17" s="9" t="inlineStr">
@@ -1524,7 +1693,7 @@
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
-          <t>0.0 ms</t>
+          <t>3676.79 ms</t>
         </is>
       </c>
       <c r="J17" s="11" t="inlineStr">
@@ -1541,32 +1710,32 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>Deduplication Engine</t>
+          <t>Semantic Analysis</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>Exact Normalized Duplicate Detection</t>
+          <t>TF-IDF Domain Keyword Ranking</t>
         </is>
       </c>
       <c r="D18" s="10" t="inlineStr">
         <is>
-          <t>Verifies that duplicate questions with minor case or punctuation variations are caught immediately.</t>
+          <t>Verifies statistical term-frequency scoring to rank high-value domain concepts.</t>
         </is>
       </c>
       <c r="E18" s="10" t="inlineStr">
         <is>
-          <t>Identical question string with different casing/punctuation</t>
+          <t>3 domain sentences about neural network architectures</t>
         </is>
       </c>
       <c r="F18" s="10" t="inlineStr">
         <is>
-          <t>is_duplicate: True, Reason identifying identical question</t>
+          <t>Top ranked terms include 'neural' and 'networks'</t>
         </is>
       </c>
       <c r="G18" s="10" t="inlineStr">
         <is>
-          <t>is_duplicate: True, Reason: 'Identical question to FAQ #1'</t>
+          <t>Identified vocabulary features: ['convolutional', 'data', 'deep', 'image', 'learning']</t>
         </is>
       </c>
       <c r="H18" s="9" t="inlineStr">
@@ -1593,32 +1762,32 @@
       </c>
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>Deduplication Engine</t>
+          <t>Semantic Analysis</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>Cosine Semantic Paraphrase Deduplication</t>
+          <t>Stopword Filtering in Feature Extraction</t>
         </is>
       </c>
       <c r="D19" s="10" t="inlineStr">
         <is>
-          <t>Verifies that paraphrased questions sharing semantic vocabulary above threshold are detected.</t>
+          <t>Ensures common grammatical stopwords (the, is, at, which) are excluded from topic extraction.</t>
         </is>
       </c>
       <c r="E19" s="10" t="inlineStr">
         <is>
-          <t>Paraphrased question with 75% lexical and n-gram overlap</t>
+          <t>Stopword-heavy sentence</t>
         </is>
       </c>
       <c r="F19" s="10" t="inlineStr">
         <is>
-          <t>is_duplicate: True via TF-IDF cosine similarity matrix</t>
+          <t>Stopwords pruned, only content words ('center', 'document', 'revolves') retained</t>
         </is>
       </c>
       <c r="G19" s="10" t="inlineStr">
         <is>
-          <t>is_duplicate: True, Reason: 'Identical answer to FAQ #1'</t>
+          <t>Retained keywords: ['center', 'document', 'revolves']</t>
         </is>
       </c>
       <c r="H19" s="9" t="inlineStr">
@@ -1645,32 +1814,32 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>Deduplication Engine</t>
+          <t>Semantic Analysis</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>Distinct Questions Preservation (Zero False Positives)</t>
+          <t>Part-of-Speech (POS) Linguistic Tagging</t>
         </is>
       </c>
       <c r="D20" s="10" t="inlineStr">
         <is>
-          <t>Verifies that distinct questions on different topics are never falsely flagged as duplicates.</t>
+          <t>Verifies linguistic noun and verb phrase tagging for question target identification.</t>
         </is>
       </c>
       <c r="E20" s="10" t="inlineStr">
         <is>
-          <t>Topic A (Submission deadline) vs Topic B (Font sizing)</t>
+          <t>Sentence: 'Offline AI models generate grounded FAQs.'</t>
         </is>
       </c>
       <c r="F20" s="10" t="inlineStr">
         <is>
-          <t>is_duplicate: False (Preserve unique FAQ)</t>
+          <t>POS sequence contains NOUN and VERB tags</t>
         </is>
       </c>
       <c r="G20" s="10" t="inlineStr">
         <is>
-          <t>is_duplicate: False, preserved successfully</t>
+          <t>Tagged POS elements: ['PROPN', 'PROPN', 'NOUN', 'VERB', 'VERB', 'PROPN', 'PUNCT']</t>
         </is>
       </c>
       <c r="H20" s="9" t="inlineStr">
@@ -1680,7 +1849,7 @@
       </c>
       <c r="I20" s="8" t="inlineStr">
         <is>
-          <t>6.98 ms</t>
+          <t>371.8 ms</t>
         </is>
       </c>
       <c r="J20" s="11" t="inlineStr">
@@ -1697,32 +1866,32 @@
       </c>
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>Deduplication Engine</t>
+          <t>Semantic Analysis</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>Identical Answer Content Deduplication</t>
+          <t>Lexical Root Frequency Distribution</t>
         </is>
       </c>
       <c r="D21" s="10" t="inlineStr">
         <is>
-          <t>Verifies that different questions resulting in identical factual answers are detected to prevent redundancy.</t>
+          <t>Verifies word frequency token count mapping across ingested text passages.</t>
         </is>
       </c>
       <c r="E21" s="10" t="inlineStr">
         <is>
-          <t>Two different question formulations yielding identical answer body</t>
+          <t>3 sentences repeating 'Ollama' 3 times</t>
         </is>
       </c>
       <c r="F21" s="10" t="inlineStr">
         <is>
-          <t>is_duplicate: True to prevent duplicate knowledge in FAQ vault</t>
+          <t>Frequency of 'ollama' == 3</t>
         </is>
       </c>
       <c r="G21" s="10" t="inlineStr">
         <is>
-          <t>is_duplicate: True, Reason: 'Identical answer to FAQ #1'</t>
+          <t>Word count for 'ollama': 3</t>
         </is>
       </c>
       <c r="H21" s="9" t="inlineStr">
@@ -1749,32 +1918,32 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>Export Engine</t>
+          <t>Generator &amp; Question Types</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>Microsoft Word (.DOCX) Export Generation</t>
+          <t>End-to-End Raw Text-to-FAQ Generation</t>
         </is>
       </c>
       <c r="D22" s="10" t="inlineStr">
         <is>
-          <t>Verifies valid DOCX byte generation with custom titles, metadata tags, and Q&amp;A blocks.</t>
+          <t>Executes the full NLP pipeline on a raw text block, producing verified question-answer pairs with page citations.</t>
         </is>
       </c>
       <c r="E22" s="10" t="inlineStr">
         <is>
-          <t>FAQ records for export to DOCX</t>
+          <t>3-sentence Capstone Guidelines text block</t>
         </is>
       </c>
       <c r="F22" s="10" t="inlineStr">
         <is>
-          <t>Valid .docx file generated (&gt; 1 KB, readable structure)</t>
+          <t>Generated FAQs with question, answer, category, and verification status</t>
         </is>
       </c>
       <c r="G22" s="10" t="inlineStr">
         <is>
-          <t>Generated DOCX size: 36710 bytes</t>
+          <t>Generated 1 verified FAQ(s)</t>
         </is>
       </c>
       <c r="H22" s="9" t="inlineStr">
@@ -1784,7 +1953,7 @@
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
-          <t>45.52 ms</t>
+          <t>11544.4 ms</t>
         </is>
       </c>
       <c r="J22" s="11" t="inlineStr">
@@ -1801,32 +1970,32 @@
       </c>
       <c r="B23" s="10" t="inlineStr">
         <is>
-          <t>Export Engine</t>
+          <t>Generator &amp; Question Types</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Plain Text (.TXT) Export Generation</t>
+          <t>Factual Question Type Classification &amp; Grounding</t>
         </is>
       </c>
       <c r="D23" s="10" t="inlineStr">
         <is>
-          <t>Verifies UTF-8 plain text export format with numbered Q&amp;A pairs and metadata.</t>
+          <t>Verifies generation and grounding of direct factual questions ('What is...', 'When is...').</t>
         </is>
       </c>
       <c r="E23" s="10" t="inlineStr">
         <is>
-          <t>FAQ records for export to TXT</t>
+          <t>Factual query on symposium date and venue</t>
         </is>
       </c>
       <c r="F23" s="10" t="inlineStr">
         <is>
-          <t>Formatted text with headers, numbered Q1/A1 pairs, and page metadata</t>
+          <t>Verified grounding with exact date (August 14) and venue matching</t>
         </is>
       </c>
       <c r="G23" s="10" t="inlineStr">
         <is>
-          <t>Generated plain text (195 chars)</t>
+          <t>Status: verified, Confidence: 0.98</t>
         </is>
       </c>
       <c r="H23" s="9" t="inlineStr">
@@ -1836,7 +2005,7 @@
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
-          <t>3.01 ms</t>
+          <t>0.0 ms</t>
         </is>
       </c>
       <c r="J23" s="11" t="inlineStr">
@@ -1853,32 +2022,32 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>API &amp; Infrastructure</t>
+          <t>Generator &amp; Question Types</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>Ollama Client Initialization &amp; Endpoint Check</t>
+          <t>Procedural Question Type Classification &amp; Grounding</t>
         </is>
       </c>
       <c r="D24" s="10" t="inlineStr">
         <is>
-          <t>Verifies Ollama client configures correct model 'qwen2.5:3b' and local base URL.</t>
+          <t>Verifies generation and grounding of step-by-step procedural questions ('How to...', 'What steps...').</t>
         </is>
       </c>
       <c r="E24" s="10" t="inlineStr">
         <is>
-          <t>OllamaClient() instantiation</t>
+          <t>Procedural workflow instruction steps</t>
         </is>
       </c>
       <c r="F24" s="10" t="inlineStr">
         <is>
-          <t>Target model set to 'qwen2.5:3b' and URL set to 'http://localhost:11434'</t>
+          <t>Step-by-step procedure verified against source passage</t>
         </is>
       </c>
       <c r="G24" s="10" t="inlineStr">
         <is>
-          <t>Model: qwen2.5:3b, Base URL: http://localhost:11434</t>
+          <t>Status: verified, Confidence: 0.99</t>
         </is>
       </c>
       <c r="H24" s="9" t="inlineStr">
@@ -1905,45 +2074,1085 @@
       </c>
       <c r="B25" s="10" t="inlineStr">
         <is>
+          <t>Generator &amp; Question Types</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Definitional Question Type Classification &amp; Grounding</t>
+        </is>
+      </c>
+      <c r="D25" s="10" t="inlineStr">
+        <is>
+          <t>Verifies generation and grounding of conceptual definition questions ('What does X mean?').</t>
+        </is>
+      </c>
+      <c r="E25" s="10" t="inlineStr">
+        <is>
+          <t>Concept definition sentence</t>
+        </is>
+      </c>
+      <c r="F25" s="10" t="inlineStr">
+        <is>
+          <t>Status: verified with high confidence definition matching</t>
+        </is>
+      </c>
+      <c r="G25" s="10" t="inlineStr">
+        <is>
+          <t>Status: verified, Confidence: 0.99</t>
+        </is>
+      </c>
+      <c r="H25" s="9" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="I25" s="8" t="inlineStr">
+        <is>
+          <t>0.0 ms</t>
+        </is>
+      </c>
+      <c r="J25" s="11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>TC21</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t>Generator &amp; Question Types</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Evaluation / Criterion Question Type Classification</t>
+        </is>
+      </c>
+      <c r="D26" s="10" t="inlineStr">
+        <is>
+          <t>Verifies criteria and grading requirement FAQ extraction ('What are the criteria for passing?').</t>
+        </is>
+      </c>
+      <c r="E26" s="10" t="inlineStr">
+        <is>
+          <t>Passage with dual percentage thresholds (70% and 75%)</t>
+        </is>
+      </c>
+      <c r="F26" s="10" t="inlineStr">
+        <is>
+          <t>Dual thresholds verified with numbers_grounded=True</t>
+        </is>
+      </c>
+      <c r="G26" s="10" t="inlineStr">
+        <is>
+          <t>Status: verified, Numbers Grounded: True</t>
+        </is>
+      </c>
+      <c r="H26" s="9" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="I26" s="8" t="inlineStr">
+        <is>
+          <t>0.0 ms</t>
+        </is>
+      </c>
+      <c r="J26" s="11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>TC22</t>
+        </is>
+      </c>
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>Generator &amp; Question Types</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>Quantitative &amp; Metric Question Grounding</t>
+        </is>
+      </c>
+      <c r="D27" s="10" t="inlineStr">
+        <is>
+          <t>Verifies strict number preservation in numerical questions (font size 14, 1.5 spacing, 20 minutes).</t>
+        </is>
+      </c>
+      <c r="E27" s="10" t="inlineStr">
+        <is>
+          <t>Quantitative passage with '20 minutes' and '5 minutes'</t>
+        </is>
+      </c>
+      <c r="F27" s="10" t="inlineStr">
+        <is>
+          <t>Both numbers confirmed present in source context</t>
+        </is>
+      </c>
+      <c r="G27" s="10" t="inlineStr">
+        <is>
+          <t>Status: verified, Confidence: 0.98</t>
+        </is>
+      </c>
+      <c r="H27" s="9" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="I27" s="8" t="inlineStr">
+        <is>
+          <t>0.0 ms</t>
+        </is>
+      </c>
+      <c r="J27" s="11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>TC23</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>Verification Engine</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>Verbatim Factual Grounding Verification</t>
+        </is>
+      </c>
+      <c r="D28" s="10" t="inlineStr">
+        <is>
+          <t>Verifies that an answer derived directly from source passage is marked 'verified' with high confidence.</t>
+        </is>
+      </c>
+      <c r="E28" s="10" t="inlineStr">
+        <is>
+          <t>Passage: 'Chapter headings must be formatted in 14 pt bold t...'</t>
+        </is>
+      </c>
+      <c r="F28" s="10" t="inlineStr">
+        <is>
+          <t>status: 'verified', confidence &gt;= 0.85, needs_review: False</t>
+        </is>
+      </c>
+      <c r="G28" s="10" t="inlineStr">
+        <is>
+          <t>status: 'verified', confidence: 0.99, excerpt located</t>
+        </is>
+      </c>
+      <c r="H28" s="9" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="I28" s="8" t="inlineStr">
+        <is>
+          <t>0.0 ms</t>
+        </is>
+      </c>
+      <c r="J28" s="11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t>TC24</t>
+        </is>
+      </c>
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>Verification Engine</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>Hallucinated Numerical Detection</t>
+        </is>
+      </c>
+      <c r="D29" s="10" t="inlineStr">
+        <is>
+          <t>Validates that when an answer introduces fictitious numbers not in source, verification flags it for review.</t>
+        </is>
+      </c>
+      <c r="E29" s="10" t="inlineStr">
+        <is>
+          <t>Source: '12 months', Answer: '36 months' (hallucination)</t>
+        </is>
+      </c>
+      <c r="F29" s="10" t="inlineStr">
+        <is>
+          <t>Flagged with needs_review=True due to unsupported numerical claim</t>
+        </is>
+      </c>
+      <c r="G29" s="10" t="inlineStr">
+        <is>
+          <t>Status: rejected, Reason: Answer contains numbers/dates not present in source: 36</t>
+        </is>
+      </c>
+      <c r="H29" s="9" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="I29" s="8" t="inlineStr">
+        <is>
+          <t>0.0 ms</t>
+        </is>
+      </c>
+      <c r="J29" s="11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>TC25</t>
+        </is>
+      </c>
+      <c r="B30" s="10" t="inlineStr">
+        <is>
+          <t>Verification Engine</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>Out-of-Domain Hallucination Detection</t>
+        </is>
+      </c>
+      <c r="D30" s="10" t="inlineStr">
+        <is>
+          <t>Verifies that completely ungrounded answers are assigned low confidence and rejected.</t>
+        </is>
+      </c>
+      <c r="E30" s="10" t="inlineStr">
+        <is>
+          <t>Biology passage vs Cryptography answer</t>
+        </is>
+      </c>
+      <c r="F30" s="10" t="inlineStr">
+        <is>
+          <t>status in ['rejected', 'needs_review'] with confidence &lt;= 0.40</t>
+        </is>
+      </c>
+      <c r="G30" s="10" t="inlineStr">
+        <is>
+          <t>status: 'rejected', confidence: 0.4</t>
+        </is>
+      </c>
+      <c r="H30" s="9" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="I30" s="8" t="inlineStr">
+        <is>
+          <t>0.0 ms</t>
+        </is>
+      </c>
+      <c r="J30" s="11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t>TC26</t>
+        </is>
+      </c>
+      <c r="B31" s="10" t="inlineStr">
+        <is>
+          <t>Verification Engine</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>Morphological Root Alignment</t>
+        </is>
+      </c>
+      <c r="D31" s="10" t="inlineStr">
+        <is>
+          <t>Verifies that morphological variants (e.g. 'formatting' vs 'format', 'require' vs 'requirement') match roots.</t>
+        </is>
+      </c>
+      <c r="E31" s="10" t="inlineStr">
+        <is>
+          <t>Passage: 'format', Answer: 'formatting'</t>
+        </is>
+      </c>
+      <c r="F31" s="10" t="inlineStr">
+        <is>
+          <t>Morphological match recognizes 'format'/'formatting' root</t>
+        </is>
+      </c>
+      <c r="G31" s="10" t="inlineStr">
+        <is>
+          <t>Status: verified, Confidence: 0.97</t>
+        </is>
+      </c>
+      <c r="H31" s="9" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="I31" s="8" t="inlineStr">
+        <is>
+          <t>0.0 ms</t>
+        </is>
+      </c>
+      <c r="J31" s="11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="9" t="inlineStr">
+        <is>
+          <t>TC27</t>
+        </is>
+      </c>
+      <c r="B32" s="10" t="inlineStr">
+        <is>
+          <t>Verification Engine</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>Empty Input Handling</t>
+        </is>
+      </c>
+      <c r="D32" s="10" t="inlineStr">
+        <is>
+          <t>Verifies that empty questions, answers, or contexts return status 'rejected' with 0.0 confidence.</t>
+        </is>
+      </c>
+      <c r="E32" s="10" t="inlineStr">
+        <is>
+          <t>Empty question, answer, and passage strings</t>
+        </is>
+      </c>
+      <c r="F32" s="10" t="inlineStr">
+        <is>
+          <t>status: 'rejected', confidence: 0.0, needs_review: True</t>
+        </is>
+      </c>
+      <c r="G32" s="10" t="inlineStr">
+        <is>
+          <t>status: 'rejected', confidence: 0.0</t>
+        </is>
+      </c>
+      <c r="H32" s="9" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="I32" s="8" t="inlineStr">
+        <is>
+          <t>0.0 ms</t>
+        </is>
+      </c>
+      <c r="J32" s="11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="9" t="inlineStr">
+        <is>
+          <t>TC28</t>
+        </is>
+      </c>
+      <c r="B33" s="10" t="inlineStr">
+        <is>
+          <t>Verification Engine</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>Supporting Source Excerpt Extraction</t>
+        </is>
+      </c>
+      <c r="D33" s="10" t="inlineStr">
+        <is>
+          <t>Verifies that the verifier pinpoints and returns the exact continuous sentence from source text.</t>
+        </is>
+      </c>
+      <c r="E33" s="10" t="inlineStr">
+        <is>
+          <t>3-sentence passage with target fact in sentence 2</t>
+        </is>
+      </c>
+      <c r="F33" s="10" t="inlineStr">
+        <is>
+          <t>Excerpt extracts 'Heading text requires 14 pt bold.'</t>
+        </is>
+      </c>
+      <c r="G33" s="10" t="inlineStr">
+        <is>
+          <t>Extracted excerpt: 'Heading text requires 14 pt bold.'</t>
+        </is>
+      </c>
+      <c r="H33" s="9" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="I33" s="8" t="inlineStr">
+        <is>
+          <t>0.0 ms</t>
+        </is>
+      </c>
+      <c r="J33" s="11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="9" t="inlineStr">
+        <is>
+          <t>TC29</t>
+        </is>
+      </c>
+      <c r="B34" s="10" t="inlineStr">
+        <is>
+          <t>Deduplication Engine</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>Exact Normalized Duplicate Detection</t>
+        </is>
+      </c>
+      <c r="D34" s="10" t="inlineStr">
+        <is>
+          <t>Verifies that duplicate questions with minor case or punctuation variations are caught immediately.</t>
+        </is>
+      </c>
+      <c r="E34" s="10" t="inlineStr">
+        <is>
+          <t>Identical question string with different casing/punctuation</t>
+        </is>
+      </c>
+      <c r="F34" s="10" t="inlineStr">
+        <is>
+          <t>is_duplicate: True, Reason identifying identical question</t>
+        </is>
+      </c>
+      <c r="G34" s="10" t="inlineStr">
+        <is>
+          <t>is_duplicate: True, Reason: 'Identical question to FAQ #1'</t>
+        </is>
+      </c>
+      <c r="H34" s="9" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="I34" s="8" t="inlineStr">
+        <is>
+          <t>0.0 ms</t>
+        </is>
+      </c>
+      <c r="J34" s="11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="9" t="inlineStr">
+        <is>
+          <t>TC30</t>
+        </is>
+      </c>
+      <c r="B35" s="10" t="inlineStr">
+        <is>
+          <t>Deduplication Engine</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>Cosine Semantic Paraphrase Deduplication</t>
+        </is>
+      </c>
+      <c r="D35" s="10" t="inlineStr">
+        <is>
+          <t>Verifies that paraphrased questions sharing semantic vocabulary above threshold are detected.</t>
+        </is>
+      </c>
+      <c r="E35" s="10" t="inlineStr">
+        <is>
+          <t>Paraphrased question with 75% lexical and n-gram overlap</t>
+        </is>
+      </c>
+      <c r="F35" s="10" t="inlineStr">
+        <is>
+          <t>is_duplicate: True via TF-IDF cosine similarity matrix</t>
+        </is>
+      </c>
+      <c r="G35" s="10" t="inlineStr">
+        <is>
+          <t>is_duplicate: True, Reason: 'Identical answer to FAQ #1'</t>
+        </is>
+      </c>
+      <c r="H35" s="9" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="I35" s="8" t="inlineStr">
+        <is>
+          <t>0.0 ms</t>
+        </is>
+      </c>
+      <c r="J35" s="11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="9" t="inlineStr">
+        <is>
+          <t>TC31</t>
+        </is>
+      </c>
+      <c r="B36" s="10" t="inlineStr">
+        <is>
+          <t>Deduplication Engine</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>Distinct Questions Preservation (Zero False Positives)</t>
+        </is>
+      </c>
+      <c r="D36" s="10" t="inlineStr">
+        <is>
+          <t>Verifies that distinct questions on different topics are never falsely flagged as duplicates.</t>
+        </is>
+      </c>
+      <c r="E36" s="10" t="inlineStr">
+        <is>
+          <t>Topic A (Submission deadline) vs Topic B (Font sizing)</t>
+        </is>
+      </c>
+      <c r="F36" s="10" t="inlineStr">
+        <is>
+          <t>is_duplicate: False (Preserve unique FAQ)</t>
+        </is>
+      </c>
+      <c r="G36" s="10" t="inlineStr">
+        <is>
+          <t>is_duplicate: False, preserved successfully</t>
+        </is>
+      </c>
+      <c r="H36" s="9" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="I36" s="8" t="inlineStr">
+        <is>
+          <t>0.0 ms</t>
+        </is>
+      </c>
+      <c r="J36" s="11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="9" t="inlineStr">
+        <is>
+          <t>TC32</t>
+        </is>
+      </c>
+      <c r="B37" s="10" t="inlineStr">
+        <is>
+          <t>Deduplication Engine</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>Identical Answer Content Deduplication</t>
+        </is>
+      </c>
+      <c r="D37" s="10" t="inlineStr">
+        <is>
+          <t>Verifies that different questions resulting in identical factual answers are detected to prevent redundancy.</t>
+        </is>
+      </c>
+      <c r="E37" s="10" t="inlineStr">
+        <is>
+          <t>Two different question formulations yielding identical answer body</t>
+        </is>
+      </c>
+      <c r="F37" s="10" t="inlineStr">
+        <is>
+          <t>is_duplicate: True to prevent duplicate knowledge in FAQ vault</t>
+        </is>
+      </c>
+      <c r="G37" s="10" t="inlineStr">
+        <is>
+          <t>is_duplicate: True, Reason: 'Identical answer to FAQ #1'</t>
+        </is>
+      </c>
+      <c r="H37" s="9" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="I37" s="8" t="inlineStr">
+        <is>
+          <t>0.0 ms</t>
+        </is>
+      </c>
+      <c r="J37" s="11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="9" t="inlineStr">
+        <is>
+          <t>TC33</t>
+        </is>
+      </c>
+      <c r="B38" s="10" t="inlineStr">
+        <is>
+          <t>Export Engine</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>Microsoft Word (.DOCX) Export Generation</t>
+        </is>
+      </c>
+      <c r="D38" s="10" t="inlineStr">
+        <is>
+          <t>Verifies valid DOCX byte generation with custom titles, metadata tags, and Q&amp;A blocks.</t>
+        </is>
+      </c>
+      <c r="E38" s="10" t="inlineStr">
+        <is>
+          <t>FAQ records for export to DOCX</t>
+        </is>
+      </c>
+      <c r="F38" s="10" t="inlineStr">
+        <is>
+          <t>Valid .docx file generated (&gt; 1 KB, readable structure)</t>
+        </is>
+      </c>
+      <c r="G38" s="10" t="inlineStr">
+        <is>
+          <t>Generated DOCX size: 36710 bytes</t>
+        </is>
+      </c>
+      <c r="H38" s="9" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="I38" s="8" t="inlineStr">
+        <is>
+          <t>46.28 ms</t>
+        </is>
+      </c>
+      <c r="J38" s="11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="9" t="inlineStr">
+        <is>
+          <t>TC34</t>
+        </is>
+      </c>
+      <c r="B39" s="10" t="inlineStr">
+        <is>
+          <t>Export Engine</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>Plain Text (.TXT) Export Generation</t>
+        </is>
+      </c>
+      <c r="D39" s="10" t="inlineStr">
+        <is>
+          <t>Verifies UTF-8 plain text export format with numbered Q&amp;A pairs and metadata.</t>
+        </is>
+      </c>
+      <c r="E39" s="10" t="inlineStr">
+        <is>
+          <t>FAQ records for export to TXT</t>
+        </is>
+      </c>
+      <c r="F39" s="10" t="inlineStr">
+        <is>
+          <t>Formatted text with headers, numbered Q1/A1 pairs, and page metadata</t>
+        </is>
+      </c>
+      <c r="G39" s="10" t="inlineStr">
+        <is>
+          <t>Generated plain text (195 chars)</t>
+        </is>
+      </c>
+      <c r="H39" s="9" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="I39" s="8" t="inlineStr">
+        <is>
+          <t>9.32 ms</t>
+        </is>
+      </c>
+      <c r="J39" s="11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="9" t="inlineStr">
+        <is>
+          <t>TC35</t>
+        </is>
+      </c>
+      <c r="B40" s="10" t="inlineStr">
+        <is>
           <t>API &amp; Infrastructure</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr">
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>Ollama Client Initialization &amp; Endpoint Check</t>
+        </is>
+      </c>
+      <c r="D40" s="10" t="inlineStr">
+        <is>
+          <t>Verifies Ollama client configures correct model 'qwen2.5:3b' and local base URL.</t>
+        </is>
+      </c>
+      <c r="E40" s="10" t="inlineStr">
+        <is>
+          <t>OllamaClient() instantiation</t>
+        </is>
+      </c>
+      <c r="F40" s="10" t="inlineStr">
+        <is>
+          <t>Target model set to 'qwen2.5:3b' and URL set to 'http://localhost:11434'</t>
+        </is>
+      </c>
+      <c r="G40" s="10" t="inlineStr">
+        <is>
+          <t>Model: qwen2.5:3b, Base URL: http://localhost:11434</t>
+        </is>
+      </c>
+      <c r="H40" s="9" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="I40" s="8" t="inlineStr">
+        <is>
+          <t>0.0 ms</t>
+        </is>
+      </c>
+      <c r="J40" s="11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="9" t="inlineStr">
+        <is>
+          <t>TC36</t>
+        </is>
+      </c>
+      <c r="B41" s="10" t="inlineStr">
+        <is>
+          <t>API &amp; Infrastructure</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
         <is>
           <t>SQLite Database Schema &amp; Model Validation</t>
         </is>
       </c>
-      <c r="D25" s="10" t="inlineStr">
+      <c r="D41" s="10" t="inlineStr">
         <is>
           <t>Validates SQLAlchemy models 'Document' and 'FAQ' with citation, category, and review fields.</t>
         </is>
       </c>
-      <c r="E25" s="10" t="inlineStr">
+      <c r="E41" s="10" t="inlineStr">
         <is>
           <t>SQLAlchemy table column definitions</t>
         </is>
       </c>
-      <c r="F25" s="10" t="inlineStr">
+      <c r="F41" s="10" t="inlineStr">
         <is>
           <t>FAQ table contains columns: ['id', 'question', 'answer', 'category', 'source_pages', 'verification_status', 'needs_review']</t>
         </is>
       </c>
-      <c r="G25" s="10" t="inlineStr">
+      <c r="G41" s="10" t="inlineStr">
         <is>
           <t>All 7 required columns present in schema</t>
         </is>
       </c>
-      <c r="H25" s="9" t="inlineStr">
-        <is>
-          <t>100.0%</t>
-        </is>
-      </c>
-      <c r="I25" s="8" t="inlineStr">
-        <is>
-          <t>0.0 ms</t>
-        </is>
-      </c>
-      <c r="J25" s="11" t="inlineStr">
+      <c r="H41" s="9" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="I41" s="8" t="inlineStr">
+        <is>
+          <t>477.31 ms</t>
+        </is>
+      </c>
+      <c r="J41" s="11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="9" t="inlineStr">
+        <is>
+          <t>TC37</t>
+        </is>
+      </c>
+      <c r="B42" s="10" t="inlineStr">
+        <is>
+          <t>Web Ingestion Engine</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>Web URL Normalization &amp; SSRF Defense</t>
+        </is>
+      </c>
+      <c r="D42" s="10" t="inlineStr">
+        <is>
+          <t>Verifies URL scheme auto-prefixing and blocking of private/loopback IP addresses.</t>
+        </is>
+      </c>
+      <c r="E42" s="10" t="inlineStr">
+        <is>
+          <t>URL normalization: 'wikipedia.org/wiki/Robotics' &amp; SSRF test: '127.0.0.1'</t>
+        </is>
+      </c>
+      <c r="F42" s="10" t="inlineStr">
+        <is>
+          <t>Auto-prefixed https:// and ValueError for internal IP hosts</t>
+        </is>
+      </c>
+      <c r="G42" s="10" t="inlineStr">
+        <is>
+          <t>Normalized: 'https://wikipedia.org/wiki/Robotics', SSRF Blocked: True</t>
+        </is>
+      </c>
+      <c r="H42" s="9" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="I42" s="8" t="inlineStr">
+        <is>
+          <t>0.0 ms</t>
+        </is>
+      </c>
+      <c r="J42" s="11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="9" t="inlineStr">
+        <is>
+          <t>TC38</t>
+        </is>
+      </c>
+      <c r="B43" s="10" t="inlineStr">
+        <is>
+          <t>Web Ingestion Engine</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>HTML DOM Sanitization &amp; Noise Elimination</t>
+        </is>
+      </c>
+      <c r="D43" s="10" t="inlineStr">
+        <is>
+          <t>Verifies stripping of script, style, navigation, footer, and cookie banner tags.</t>
+        </is>
+      </c>
+      <c r="E43" s="10" t="inlineStr">
+        <is>
+          <t>HTML with embedded script, style, nav, cookie banner, and article paragraphs</t>
+        </is>
+      </c>
+      <c r="F43" s="10" t="inlineStr">
+        <is>
+          <t>Scripts, nav, footer, and ads stripped; clean article paragraphs retained</t>
+        </is>
+      </c>
+      <c r="G43" s="10" t="inlineStr">
+        <is>
+          <t>Scripts Stripped: True, Nav Stripped: True, Cookies Stripped: True, Content Retained: True</t>
+        </is>
+      </c>
+      <c r="H43" s="9" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="I43" s="8" t="inlineStr">
+        <is>
+          <t>6.0 ms</t>
+        </is>
+      </c>
+      <c r="J43" s="11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="9" t="inlineStr">
+        <is>
+          <t>TC39</t>
+        </is>
+      </c>
+      <c r="B44" s="10" t="inlineStr">
+        <is>
+          <t>Web Ingestion Engine</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>Heading-Aware Webpage Section Partitioning</t>
+        </is>
+      </c>
+      <c r="D44" s="10" t="inlineStr">
+        <is>
+          <t>Verifies web content is partitioned into structured sections matching DocumentProcessor pages.</t>
+        </is>
+      </c>
+      <c r="E44" s="10" t="inlineStr">
+        <is>
+          <t>3-section technical article with H1 and H2 tags</t>
+        </is>
+      </c>
+      <c r="F44" s="10" t="inlineStr">
+        <is>
+          <t>3 discrete section pages with accurate headings and word counts</t>
+        </is>
+      </c>
+      <c r="G44" s="10" t="inlineStr">
+        <is>
+          <t>Sections Count: 3, Headings Detected: 3</t>
+        </is>
+      </c>
+      <c r="H44" s="9" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="I44" s="8" t="inlineStr">
+        <is>
+          <t>1.04 ms</t>
+        </is>
+      </c>
+      <c r="J44" s="11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="9" t="inlineStr">
+        <is>
+          <t>TC40</t>
+        </is>
+      </c>
+      <c r="B45" s="10" t="inlineStr">
+        <is>
+          <t>Web Ingestion Engine</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>Webpage-Grounded FAQ Citation &amp; Fact Verification</t>
+        </is>
+      </c>
+      <c r="D45" s="10" t="inlineStr">
+        <is>
+          <t>Verifies that FAQ questions generated from a webpage are factually grounded and cite exact section headings.</t>
+        </is>
+      </c>
+      <c r="E45" s="10" t="inlineStr">
+        <is>
+          <t>Webpage section text and candidate question/answer pair</t>
+        </is>
+      </c>
+      <c r="F45" s="10" t="inlineStr">
+        <is>
+          <t>Grounding verified = True, confidence &gt;= 90%, source section retained</t>
+        </is>
+      </c>
+      <c r="G45" s="10" t="inlineStr">
+        <is>
+          <t>Status: verified, Confidence: 99.0%, Section: 'Control Plane Components'</t>
+        </is>
+      </c>
+      <c r="H45" s="9" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="I45" s="8" t="inlineStr">
+        <is>
+          <t>3.07 ms</t>
+        </is>
+      </c>
+      <c r="J45" s="11" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>

</xml_diff>